<commit_message>
godot: retours de partie sur l'ouverture : champ, boue, Trafic en jaune, rue déjà déblayée
Demande de l'auteur (partie jouée en direct) : le guide dit « un champ » sans les ponts, la fiche du champ ne répète plus le bas, la Ville s'entoure pour aller voir la boue, l'anneau du rail passe en jaune, la rue déblayée n'est plus proposée. 9 essais à 0 échec, sauvegarde 92 comme avant ; textes ajoutés au tableau de l'auteur.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prototype/Textes des premières minutes.xlsx
+++ b/Prototype/Textes des premières minutes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premières minutes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Premières minutes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -891,13 +891,13 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>[3] ponts coupés : elles restent sur leur rive. Cliquez sur un lieu pour les abriter.</t>
+          <t>Trouvez un champ où poser des containers pour les loger.</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr"/>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Ne désigne aucun champ.</t>
+          <t>Ne désigne aucun champ. Les ponts coupés ne sont plus dits ici (2026-10-06).</t>
         </is>
       </c>
     </row>
@@ -914,13 +914,13 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Un camp demande un terrain nu.</t>
+          <t>(retiré le 2026-10-06)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr"/>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Ne s'affiche qu'après 3 lieux ouverts sans avoir ouvert de champ.</t>
+          <t>Inutile depuis que le guide dit « un champ ».</t>
         </is>
       </c>
     </row>
@@ -1070,11 +1070,15 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Jusqu'à [238] personnes · [119] containers</t>
+          <t>(retiré le 2026-10-06)</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
-      <c r="E31" s="7" t="inlineStr"/>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Prix, abrités et nourris sont dans les conséquences du bas.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="19" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -1089,11 +1093,15 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>⚠ Il ne sera plus jamais cultivé.</t>
+          <t>(retiré le 2026-10-06)</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr"/>
-      <c r="E32" s="7" t="inlineStr"/>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Idem.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="19" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -1884,13 +1892,13 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>La boue bloque le chemin jusqu'au pont : déblayez-le pendant le chantier.</t>
+          <t>La boue bloque le chemin jusqu'au pont. Revenez sur la ville pour la voir, et déblayez pendant le chantier.</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr"/>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>Ne nomme pas la rue : le joueur la cherche.</t>
+          <t>Ne nomme pas la rue. La tuile Ville s'entoure en jaune tant qu'on n'y est pas revenu.</t>
         </is>
       </c>
     </row>
@@ -2021,11 +2029,15 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Encore [12] rues sous la boue : Trafic propose de tout déblayer d'un coup.</t>
+          <t>Encore [12] rues sous la boue : ouvrez Trafic pour tout déblayer d'un coup.</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr"/>
-      <c r="E81" s="7" t="inlineStr"/>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>La tuile Trafic s'entoure en jaune.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="34" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
@@ -3165,7 +3177,7 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Un premier lieu à relever</t>
+          <t>Un premier lieu à relever   /   rue déjà déblayée : Reconstruisons quelque chose pour les habitants</t>
         </is>
       </c>
       <c r="D142" s="6" t="inlineStr"/>
@@ -3185,6 +3197,8 @@
       <c r="C143" s="4" t="inlineStr">
         <is>
           <t>Rue des Forgerons envasée, [43] logements inhabitables à côté. La prochaine crue y mettrait [5,1] m d'eau. Par où commencer ?
+[6] autres îlots attendent. La caisse ne les relèvera pas tous.
+— rue déjà déblayée : [Maisons des Forgerons] : [43] logements inhabitables. La prochaine crue y mettrait [5,1] m d'eau.
 [6] autres îlots attendent. La caisse ne les relèvera pas tous.</t>
         </is>
       </c>
@@ -3204,7 +3218,8 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>① Déblayer la rue   ·   ② Relever les logements · [43] personnes peuvent rentrer</t>
+          <t>① Déblayer la rue   ·   ② Relever les logements · [43] personnes peuvent rentrer
+— rue déjà déblayée : Relever [Maisons des Forgerons] · [43] personnes peuvent rentrer</t>
         </is>
       </c>
       <c r="D144" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
godot: le joueur choisit l'îlot à relever, et ceux qui rentrent emportent leurs containers
Demande de l'auteur : après le pont, le guide ne désigne plus les Forgerons ; la fiche d'un îlot sinistré dit combien quittent le camp ; 43 rentrés = 21 containers retirés, le dernier camp posé se vide d'abord ; titre « Relogement » retiré. 9 essais à 0 échec, sauvegarde 92 comme avant.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prototype/Textes des premières minutes.xlsx
+++ b/Prototype/Textes des premières minutes.xlsx
@@ -1051,11 +1051,15 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Relogement</t>
+          <t>(retiré le 2026-10-06)</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr"/>
-      <c r="E30" s="7" t="inlineStr"/>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Le bouton « Installer… » suffit.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="19" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -3177,11 +3181,15 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Un premier lieu à relever   /   rue déjà déblayée : Reconstruisons quelque chose pour les habitants</t>
+          <t>Le pont est rouvert</t>
         </is>
       </c>
       <c r="D142" s="6" t="inlineStr"/>
-      <c r="E142" s="7" t="inlineStr"/>
+      <c r="E142" s="7" t="inlineStr">
+        <is>
+          <t>Ne désigne aucun îlot : le joueur choisit (2026-10-06).</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="49" customHeight="1">
       <c r="A143" s="4" t="inlineStr">
@@ -3196,10 +3204,8 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Rue des Forgerons envasée, [43] logements inhabitables à côté. La prochaine crue y mettrait [5,1] m d'eau. Par où commencer ?
-[6] autres îlots attendent. La caisse ne les relèvera pas tous.
-— rue déjà déblayée : [Maisons des Forgerons] : [43] logements inhabitables. La prochaine crue y mettrait [5,1] m d'eau.
-[6] autres îlots attendent. La caisse ne les relèvera pas tous.</t>
+          <t>[238] personnes vivent encore dans les containers. Choisissez un îlot à reconstruire.
+[7] îlots attendent. La caisse ne les relèvera pas tous.</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr"/>
@@ -3218,12 +3224,15 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>① Déblayer la rue   ·   ② Relever les logements · [43] personnes peuvent rentrer
-— rue déjà déblayée : Relever [Maisons des Forgerons] · [43] personnes peuvent rentrer</t>
+          <t>(retiré le 2026-10-06)</t>
         </is>
       </c>
       <c r="D144" s="6" t="inlineStr"/>
-      <c r="E144" s="7" t="inlineStr"/>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>Plus de bouton : on clique sur l'îlot dans la ville.</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="94" customHeight="1">
       <c r="A145" s="4" t="inlineStr">
@@ -3238,7 +3247,7 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>[8] bâtiments détruits, [43] logements perdus. La crue annoncée en reprendrait [100] %.
+          <t>[8] bâtiments détruits, [43] logements perdus. Relevé, [43] personnes quittent le camp. La crue annoncée en reprendrait [100] %.
 Comment le relever ?
 — bouton : Comme avant
 Autrement qu'avant : un concours, pour tous les îlots sinistrés.
@@ -3246,7 +3255,11 @@
         </is>
       </c>
       <c r="D145" s="6" t="inlineStr"/>
-      <c r="E145" s="7" t="inlineStr"/>
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>Le nombre qui quitte le camp sert à comparer les îlots.</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="19" customHeight="1">
       <c r="A146" s="4" t="inlineStr">
@@ -3300,7 +3313,7 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Laisser avancer · ×12   ·   Voir mon chantier   ·   Comparer les logements / Comparer la rue</t>
+          <t>Laisser avancer · ×12   ·   Voir mon chantier</t>
         </is>
       </c>
       <c r="D148" s="6" t="inlineStr"/>

</xml_diff>